<commit_message>
볼트 작업 사본의 07-16~09-03 개선분 반영(ia-builder·wbs·weekly-report·requirements 스크립트, 스킬 문서, meeting-agenda 스킬 추가), 볼트 frontmatter·관련 문서 흔적 제거, _output 제외
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/skills/ia-builder/samples/결과_예시.xlsx
+++ b/skills/ia-builder/samples/결과_예시.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="표지" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="사용안내" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="개정이력" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Front 정보구조도" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Admin 정보구조도" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="표지" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용안내" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개정이력" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Front 정보구조도" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin 정보구조도" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1237,7 +1237,7 @@
     <row r="5" ht="19" customHeight="1">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="B5" s="20" t="inlineStr">
@@ -1281,7 +1281,7 @@
     <row r="6" ht="19" customHeight="1">
       <c r="A6" s="22" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="B6" s="23" t="inlineStr">
@@ -1303,7 +1303,7 @@
     <row r="7" ht="19" customHeight="1">
       <c r="A7" s="24" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="B7" s="25" t="n"/>
@@ -1339,7 +1339,7 @@
     <row r="8" ht="19" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="B8" s="27" t="n"/>
@@ -1375,7 +1375,7 @@
     <row r="9" ht="19" customHeight="1">
       <c r="A9" s="24" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="B9" s="25" t="n"/>
@@ -1411,7 +1411,7 @@
     <row r="10" ht="19" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="B10" s="27" t="n"/>
@@ -1451,7 +1451,7 @@
     <row r="11" ht="19" customHeight="1">
       <c r="A11" s="22" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="B11" s="23" t="inlineStr">
@@ -1473,7 +1473,7 @@
     <row r="12" ht="19" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="B12" s="27" t="n"/>
@@ -1495,7 +1495,7 @@
     <row r="13" ht="19" customHeight="1">
       <c r="A13" s="24" t="inlineStr">
         <is>
-          <t>2.1.1</t>
+          <t>3.1.1</t>
         </is>
       </c>
       <c r="B13" s="25" t="n"/>
@@ -1531,7 +1531,7 @@
     <row r="14" ht="19" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>2.1.2</t>
+          <t>3.1.2</t>
         </is>
       </c>
       <c r="B14" s="27" t="n"/>
@@ -1575,7 +1575,7 @@
     <row r="15" ht="19" customHeight="1">
       <c r="A15" s="24" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="B15" s="25" t="n"/>
@@ -1597,7 +1597,7 @@
     <row r="16" ht="19" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>2.2.1</t>
+          <t>3.2.1</t>
         </is>
       </c>
       <c r="B16" s="27" t="n"/>
@@ -1633,7 +1633,7 @@
     <row r="17" ht="19" customHeight="1">
       <c r="A17" s="24" t="inlineStr">
         <is>
-          <t>2.2.2</t>
+          <t>3.2.2</t>
         </is>
       </c>
       <c r="B17" s="25" t="n"/>
@@ -1677,7 +1677,7 @@
     <row r="18" ht="19" customHeight="1">
       <c r="A18" s="22" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="B18" s="23" t="inlineStr">
@@ -1699,7 +1699,7 @@
     <row r="19" ht="19" customHeight="1">
       <c r="A19" s="24" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="B19" s="25" t="n"/>
@@ -1743,7 +1743,7 @@
     <row r="20" ht="19" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="B20" s="27" t="n"/>
@@ -1783,7 +1783,7 @@
     <row r="21" ht="19" customHeight="1">
       <c r="A21" s="24" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="B21" s="25" t="n"/>
@@ -1819,7 +1819,7 @@
     <row r="22" ht="19" customHeight="1">
       <c r="A22" s="22" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="B22" s="23" t="inlineStr">
@@ -1841,7 +1841,7 @@
     <row r="23" ht="19" customHeight="1">
       <c r="A23" s="24" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="B23" s="25" t="n"/>
@@ -1881,7 +1881,7 @@
     <row r="24" ht="19" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>5.2</t>
         </is>
       </c>
       <c r="B24" s="27" t="n"/>
@@ -1921,7 +1921,7 @@
     <row r="25" ht="19" customHeight="1">
       <c r="A25" s="24" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="B25" s="25" t="n"/>
@@ -1957,7 +1957,7 @@
     <row r="26" ht="19" customHeight="1">
       <c r="A26" s="22" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="B26" s="23" t="inlineStr">
@@ -1979,7 +1979,7 @@
     <row r="27" ht="19" customHeight="1">
       <c r="A27" s="24" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="B27" s="25" t="n"/>
@@ -2015,7 +2015,7 @@
     <row r="28" ht="19" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="B28" s="27" t="n"/>
@@ -2055,7 +2055,7 @@
     <row r="29" ht="19" customHeight="1">
       <c r="A29" s="24" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>6.3</t>
         </is>
       </c>
       <c r="B29" s="25" t="n"/>
@@ -2091,7 +2091,7 @@
     <row r="30" ht="19" customHeight="1">
       <c r="A30" s="22" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>7.0</t>
         </is>
       </c>
       <c r="B30" s="23" t="inlineStr">
@@ -2113,7 +2113,7 @@
     <row r="31" ht="19" customHeight="1">
       <c r="A31" s="24" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="B31" s="25" t="n"/>
@@ -2135,7 +2135,7 @@
     <row r="32" ht="19" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>6.1.1</t>
+          <t>7.1.1</t>
         </is>
       </c>
       <c r="B32" s="27" t="n"/>
@@ -2179,7 +2179,7 @@
     <row r="33" ht="19" customHeight="1">
       <c r="A33" s="24" t="inlineStr">
         <is>
-          <t>6.1.2</t>
+          <t>7.1.2</t>
         </is>
       </c>
       <c r="B33" s="25" t="n"/>
@@ -2215,7 +2215,7 @@
     <row r="34" ht="19" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>6.1.3</t>
+          <t>7.1.3</t>
         </is>
       </c>
       <c r="B34" s="27" t="n"/>
@@ -2255,7 +2255,7 @@
     <row r="35" ht="19" customHeight="1">
       <c r="A35" s="24" t="inlineStr">
         <is>
-          <t>6.1.4</t>
+          <t>7.1.4</t>
         </is>
       </c>
       <c r="B35" s="25" t="n"/>
@@ -2291,7 +2291,7 @@
     <row r="36" ht="19" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>7.2</t>
         </is>
       </c>
       <c r="B36" s="27" t="n"/>
@@ -2335,7 +2335,7 @@
     <row r="37" ht="19" customHeight="1">
       <c r="A37" s="24" t="inlineStr">
         <is>
-          <t>6.3</t>
+          <t>7.3</t>
         </is>
       </c>
       <c r="B37" s="25" t="n"/>
@@ -2375,7 +2375,7 @@
     <row r="38" ht="19" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>6.4</t>
+          <t>7.4</t>
         </is>
       </c>
       <c r="B38" s="27" t="n"/>
@@ -2411,7 +2411,7 @@
     <row r="39" ht="19" customHeight="1">
       <c r="A39" s="24" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="B39" s="25" t="n"/>
@@ -2817,7 +2817,7 @@
     <row r="5" ht="19" customHeight="1">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>A.1</t>
+          <t>A.1.0</t>
         </is>
       </c>
       <c r="B5" s="20" t="inlineStr">
@@ -2843,7 +2843,7 @@
       <c r="H5" s="32" t="n"/>
       <c r="I5" s="33" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J5" s="32" t="n"/>
@@ -2851,7 +2851,7 @@
       <c r="L5" s="32" t="n"/>
       <c r="M5" s="33" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="N5" s="32" t="n"/>
@@ -2859,7 +2859,7 @@
       <c r="P5" s="32" t="n"/>
       <c r="Q5" s="33" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="R5" s="32" t="n"/>
@@ -2869,7 +2869,7 @@
     <row r="6" ht="19" customHeight="1">
       <c r="A6" s="22" t="inlineStr">
         <is>
-          <t>A.2</t>
+          <t>A.2.0</t>
         </is>
       </c>
       <c r="B6" s="23" t="inlineStr">
@@ -2895,7 +2895,7 @@
       <c r="H6" s="34" t="n"/>
       <c r="I6" s="35" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J6" s="34" t="n"/>
@@ -2903,7 +2903,7 @@
       <c r="L6" s="34" t="n"/>
       <c r="M6" s="35" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="N6" s="34" t="n"/>
@@ -2911,7 +2911,7 @@
       <c r="P6" s="34" t="n"/>
       <c r="Q6" s="35" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="R6" s="34" t="n"/>
@@ -2921,7 +2921,7 @@
     <row r="7" ht="19" customHeight="1">
       <c r="A7" s="22" t="inlineStr">
         <is>
-          <t>A.3</t>
+          <t>A.3.0</t>
         </is>
       </c>
       <c r="B7" s="23" t="inlineStr">
@@ -2976,62 +2976,62 @@
       </c>
       <c r="H8" s="36" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="I8" s="36" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J8" s="36" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K8" s="36" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L8" s="36" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="M8" s="36" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="N8" s="36" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O8" s="36" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P8" s="36" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="Q8" s="36" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="R8" s="36" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="S8" s="36" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="T8" s="27" t="n"/>
@@ -3065,49 +3065,49 @@
       <c r="H9" s="37" t="n"/>
       <c r="I9" s="33" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J9" s="37" t="n"/>
       <c r="K9" s="33" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L9" s="37" t="n"/>
       <c r="M9" s="33" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="N9" s="33" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O9" s="33" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P9" s="33" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="Q9" s="33" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="R9" s="33" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="S9" s="33" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="T9" s="25" t="n"/>
@@ -3115,7 +3115,7 @@
     <row r="10" ht="19" customHeight="1">
       <c r="A10" s="22" t="inlineStr">
         <is>
-          <t>A.4</t>
+          <t>A.4.0</t>
         </is>
       </c>
       <c r="B10" s="23" t="inlineStr">
@@ -3141,7 +3141,7 @@
       <c r="H10" s="34" t="n"/>
       <c r="I10" s="35" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J10" s="34" t="n"/>
@@ -3149,33 +3149,33 @@
       <c r="L10" s="34" t="n"/>
       <c r="M10" s="35" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="N10" s="35" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O10" s="34" t="n"/>
       <c r="P10" s="35" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="Q10" s="35" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="R10" s="35" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="S10" s="35" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="T10" s="23" t="n"/>
@@ -3183,7 +3183,7 @@
     <row r="11" ht="19" customHeight="1">
       <c r="A11" s="22" t="inlineStr">
         <is>
-          <t>A.5</t>
+          <t>A.5.0</t>
         </is>
       </c>
       <c r="B11" s="23" t="inlineStr">
@@ -3243,29 +3243,29 @@
       <c r="L12" s="37" t="n"/>
       <c r="M12" s="36" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="N12" s="37" t="n"/>
       <c r="O12" s="37" t="n"/>
       <c r="P12" s="36" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="Q12" s="36" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="R12" s="36" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="S12" s="36" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="T12" s="27" t="n"/>
@@ -3306,22 +3306,22 @@
       <c r="O13" s="38" t="n"/>
       <c r="P13" s="40" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="Q13" s="40" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="R13" s="40" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="S13" s="40" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>O</t>
         </is>
       </c>
       <c r="T13" s="39" t="inlineStr">

</xml_diff>